<commit_message>
fix(student): correct application withdrawal routing and cast UUIDs in query
</commit_message>
<xml_diff>
--- a/campus-placement/qa/C-10-Profile-Editability-and-Immutable-Identity-Fields.xlsx
+++ b/campus-placement/qa/C-10-Profile-Editability-and-Immutable-Identity-Fields.xlsx
@@ -602,15 +602,11 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr"/>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>Automated test execution</t>
-        </is>
-      </c>
+      <c r="Q2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -683,15 +679,11 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>Automated test execution</t>
-        </is>
-      </c>
+      <c r="Q3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -764,15 +756,11 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Not Run</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr"/>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>Automated test execution</t>
-        </is>
-      </c>
+      <c r="Q4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">

</xml_diff>